<commit_message>
Ajusta o texto de Competência 2025: 2025 já fechou, fica em 2026 mesmo
Correção de linguagem: não sugerir mais mover a despesa pra 2025 (não
dá, o exercício já está encerrado). A despesa fica em 2026 mesmo — a
aba Pendências e a nota do Resumo agora deixam claro que é uma
variação de competência documentada por fornecedor pra auditoria e
para o CFO, não uma pendência de lançamento. Números idênticos, só o
texto ficou certo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019kZogLAifrFqnDpPRs6yMP
</commit_message>
<xml_diff>
--- a/entregas/Jusfy - Ajustes contabeis Jan-Jun 2026 para Syhus.xlsx
+++ b/entregas/Jusfy - Ajustes contabeis Jan-Jun 2026 para Syhus.xlsx
@@ -74,7 +74,7 @@
     <t>Folha: distratos já reconciliados pessoa a pessoa — diferença entre painel total e Realizado por pessoa, sem ação pendente</t>
   </si>
   <si>
-    <t>Competência de 2025 lançada em 2026 (exercício anterior — ponto de atenção, não é ajuste de 2026)</t>
+    <t>Competência de 2025 lançada em 2026 (exercício de 2025 já encerrado — fica em 2026; variação para auditoria)</t>
   </si>
   <si>
     <t>A mais no razão sem prova — pedir NF (aba Pendências)</t>
@@ -128,7 +128,7 @@
     <t>Despesa de ano anterior lançada no ano corrente</t>
   </si>
   <si>
-    <t>Olhar a data da nota antes de lançar: se é do ano anterior, não é despesa deste ano — lançar contra a provisão/resultado do ano dela.</t>
+    <t>A NF chegou tão atrasada que passou pro ano seguinte. Prevenção: provisionar no fechamento de dezembro o que já se sabe que vai chegar atrasado. O que já caiu em 2026 fica em 2026 (2025 já fechou) — não é pra mover; é variação de competência documentada na aba Pendências, pra auditoria e CFO.</t>
   </si>
   <si>
     <t>Provisão que nunca foi revertida (fica pendurada, duplica a despesa)</t>
@@ -155,7 +155,7 @@
     <t>15 AJUSTES — o que fecha a meta de 0,5% (o resto pode esperar)</t>
   </si>
   <si>
-    <t>Só estes 15 lançamentos, por fornecedor, já deixam os 6 meses dentro de 0,5% de diferença contra o gerencial (considerando as notas explicativas já aceitas — Pagar.me, folha e despesas de 2025, aba Resumo). As abas "O QUE FAZER" e "Provisões" trazem o resto (não muda o resultado do mês ou é de baixo impacto); a aba "Trocar de conta (sem pressa)" nem muda o resultado — pode ficar pra depois.</t>
+    <t>Só estes 15 lançamentos, por fornecedor, já deixam os 6 meses dentro de 0,5% de diferença contra o gerencial (considerando as notas explicativas já aceitas — Pagar.me, folha e competência de 2025, exercício encerrado, ver aba Resumo). As abas "O QUE FAZER" e "Provisões" trazem o resto (não muda o resultado do mês ou é de baixo impacto); a aba "Trocar de conta (sem pressa)" nem muda o resultado — pode ficar pra depois.</t>
   </si>
   <si>
     <t>Mês</t>
@@ -4574,13 +4574,13 @@
     <t>TOTAL (37 linhas)</t>
   </si>
   <si>
-    <t>Competência de 2025 — ponto de atenção (não é ajuste de 2026)</t>
-  </si>
-  <si>
-    <t>É despesa do exercício anterior (2025) que entrou na despesa de 2026. NÃO pedimos pra lançar como correção do mês — é do ano passado, não é erro de 2026. Fica registrado aqui como nota explicativa da diferença (mesmo valor na aba Resumo, seção "PADRÕES DE ERRO" e "DE ONDE VEM A DIFERENÇA").</t>
-  </si>
-  <si>
-    <t>Valor (do exercício anterior)</t>
+    <t>Competência de 2025 — variação de competência para auditoria (não é lançamento pendente)</t>
+  </si>
+  <si>
+    <t>O exercício de 2025 já está encerrado, então essa despesa fica em 2026 mesmo — não há nada a mover nem lançamento de correção a pedir da Syhus. Fica documentado aqui, por fornecedor, pra auditoria e para o CFO acompanharem a variação (mesmo valor na aba Resumo, seções "PADRÕES DE ERRO" e "DE ONDE VEM A DIFERENÇA").</t>
+  </si>
+  <si>
+    <t>Valor (competência 2025, efeito em 2026)</t>
   </si>
   <si>
     <t>Nota explicativa</t>
@@ -6283,7 +6283,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" ht="48" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="22" t="s">
         <v>35</v>
       </c>

</xml_diff>